<commit_message>
Fix: xlsx metadata and formatting
</commit_message>
<xml_diff>
--- a/public/budsjettmal.xlsx
+++ b/public/budsjettmal.xlsx
@@ -31,7 +31,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
@@ -41,7 +41,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -52,12 +52,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="002563EB"/>
         <bgColor rgb="002563EB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EFF6FF"/>
-        <bgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -109,24 +103,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,17 +490,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PENGEPRATEN.NO - MÅNEDLIG BUDSJETT</t>
@@ -510,67 +508,62 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Måned:</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Kategori</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Januar 2026</t>
+          <t>Budsjett (kr)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Faktisk (kr)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Differanse</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Merknad</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Kategori</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Budsjett (kr)</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Faktisk (kr)</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Differanse (kr)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Kommentar</t>
-        </is>
-      </c>
+          <t>INNTEKTER</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>INNTEKTER</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lønn</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>35000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Lønn</t>
+          <t xml:space="preserve">  Bonus</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>35000</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -581,40 +574,28 @@
       <c r="B8" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="9"/>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>UTGIFTER</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Leie/Husleie</t>
+          <t xml:space="preserve">  Leie</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>12000</v>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -625,9 +606,6 @@
       <c r="B12" t="n">
         <v>1000</v>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -638,9 +616,6 @@
       <c r="B13" t="n">
         <v>500</v>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -651,9 +626,6 @@
       <c r="B14" t="n">
         <v>4000</v>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -664,9 +636,6 @@
       <c r="B15" t="n">
         <v>2000</v>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -677,84 +646,56 @@
       <c r="B16" t="n">
         <v>1000</v>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Forsikring</t>
+          <t xml:space="preserve">  Annet</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>500</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Annet</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
         <v>2000</v>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="18"/>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>SUM INNTEKT</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>35000</v>
+      </c>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>SUM INNTEKT</t>
-        </is>
-      </c>
-      <c r="B20" s="5">
-        <f>SUM(B7:B8)</f>
-        <v/>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>SUM UTGIFTER</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>23500</v>
+      </c>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>SUM UTGIFTER</t>
-        </is>
-      </c>
-      <c r="B21" s="5">
-        <f>SUM(B11:B18)</f>
-        <v/>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>DISPONIBELT</t>
         </is>
       </c>
-      <c r="B22">
-        <f>B20-B21</f>
-        <v/>
-      </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="B21" s="4" t="n">
+        <v>11500</v>
+      </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -770,104 +711,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ÅRSBUDSJETT 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Måned</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Inntekt</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Utgift</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Disposable</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Inntekt (kr)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Utgift (kr)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Disponibelt (kr)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Januar</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>35000</v>
       </c>
       <c r="C4" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D4">
-        <f>B4-C4</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Februar</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>35000</v>
       </c>
       <c r="C5" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D5">
-        <f>B5-C5</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>35000</v>
       </c>
       <c r="C6" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D6">
-        <f>B6-C6</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D6" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>April</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>35000</v>
       </c>
       <c r="C7" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D7">
-        <f>B7-C7</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="8">
@@ -880,135 +823,127 @@
         <v>35000</v>
       </c>
       <c r="C8" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D8">
-        <f>B8-C8</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Juni</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>35000</v>
       </c>
       <c r="C9" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D9">
-        <f>B9-C9</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D9" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jul</t>
+          <t>Juli</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>35000</v>
       </c>
       <c r="C10" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D10">
-        <f>B10-C10</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D10" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>August</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>35000</v>
       </c>
       <c r="C11" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D11">
-        <f>B11-C11</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D11" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>September</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>35000</v>
       </c>
       <c r="C12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D12">
-        <f>B12-C12</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Okt</t>
+          <t>Oktober</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>35000</v>
       </c>
       <c r="C13" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D13">
-        <f>B13-C13</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D13" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Nov</t>
+          <t>November</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>35000</v>
       </c>
       <c r="C14" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D14">
-        <f>B14-C14</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D14" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Des</t>
+          <t>Desember</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>35000</v>
       </c>
       <c r="C15" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D15">
-        <f>B15-C15</f>
-        <v/>
+        <v>23500</v>
+      </c>
+      <c r="D15" t="n">
+        <v>11500</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1022,36 +957,43 @@
   </sheetPr>
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>GJELDSBREMS - BLI GJELDFRI RASKERE</t>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>GJELDSBREMS - BLI GJELDFRI</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Gjeld</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Rente (%)</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Minimum (kr)</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Min. betaling (kr)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Ekstra (kr)</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Måneder igjen</t>
         </is>
@@ -1105,36 +1047,43 @@
   </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>SPAREMÅL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Mål</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Beløp (kr)</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Spart (kr)</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Gjenstår (kr)</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Fremdrift (%)</t>
         </is>
@@ -1143,7 +1092,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Buffer (3 måneders forbruk)</t>
+          <t>Buffer (3 mnd)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1152,13 +1101,13 @@
       <c r="C4" t="n">
         <v>15000</v>
       </c>
-      <c r="D4">
-        <f>B4-C4</f>
-        <v/>
-      </c>
-      <c r="E4">
-        <f>C4/B4</f>
-        <v/>
+      <c r="D4" t="n">
+        <v>35000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1173,13 +1122,13 @@
       <c r="C5" t="n">
         <v>5000</v>
       </c>
-      <c r="D5">
-        <f>B5-C5</f>
-        <v/>
-      </c>
-      <c r="E5">
-        <f>C5/B5</f>
-        <v/>
+      <c r="D5" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>17%</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1194,13 +1143,13 @@
       <c r="C6" t="n">
         <v>0</v>
       </c>
-      <c r="D6">
-        <f>B6-C6</f>
-        <v/>
-      </c>
-      <c r="E6">
-        <f>C6/B6</f>
-        <v/>
+      <c r="D6" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: XML compatibility - dates, empty cells
</commit_message>
<xml_diff>
--- a/public/budsjettmal.xlsx
+++ b/public/budsjettmal.xlsx
@@ -540,10 +540,10 @@
           <t>INNTEKTER</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -582,10 +582,10 @@
           <t>UTGIFTER</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
+      <c r="B10"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -667,9 +667,9 @@
       <c r="B19" s="4" t="n">
         <v>35000</v>
       </c>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -680,9 +680,9 @@
       <c r="B20" s="3" t="n">
         <v>23500</v>
       </c>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -693,9 +693,9 @@
       <c r="B21" s="4" t="n">
         <v>11500</v>
       </c>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>